<commit_message>
Update course plans and analysis documents across multiple subjects
- Updated binary files for analysis and course plans in IHV, IKS, and ISLL departments.
- Modified markdown files to reflect changes in course availability and details, including the addition of new courses and updates to existing ones.
- Adjusted the number of courses listed in various sections to ensure accuracy.
- Added tags and CSS classes to markdown files for better categorization of courses.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/04 ISLL/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/04 ISLL/Analys/Vilande kursplaner.xlsx
@@ -5721,7 +5721,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>GIT2T6</t>
+          <t>GIT2A3</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>2021-12-21</t>
+          <t>2019-06-19</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Italienska nobelpristagare i litteratur</t>
+          <t>Italienska B: Muntlig språkfärdighet och kulturkunskap</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5761,14 +5761,14 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2T6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2A3</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>GIT2TD</t>
+          <t>GIT2T6</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Italienska A: Italiensk affärskommunikation och -kultur</t>
+          <t>Italienska nobelpristagare i litteratur</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5808,14 +5808,14 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2T6</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>GIT2TG</t>
+          <t>GIT2TD</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5845,7 +5845,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Italienska A: Kultur och samhälle, norra Italien</t>
+          <t>Italienska A: Italiensk affärskommunikation och -kultur</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -5855,14 +5855,14 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TD</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>GIT2TH</t>
+          <t>GIT2TE</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, en litterär resa i norra Italien</t>
+          <t>Italienska A: Fonetik och muntlig språkfärdighet</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5902,14 +5902,14 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TE</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>GIT2TJ</t>
+          <t>GIT2TG</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, en litterär resa på de italienska öarna</t>
+          <t>Italienska A: Kultur och samhälle, norra Italien</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5949,14 +5949,14 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TG</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>GIT2TK</t>
+          <t>GIT2TH</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Italienska A: Kultur och samhälle, de italienska öarna</t>
+          <t>Italienska A: Textanalys, en litterär resa i norra Italien</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5996,14 +5996,14 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TH</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>GIT2TM</t>
+          <t>GIT2TJ</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -6033,7 +6033,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, en litterär resa i södra Italien</t>
+          <t>Italienska A: Textanalys, en litterär resa på de italienska öarna</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -6043,14 +6043,14 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TJ</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>GIT2TN</t>
+          <t>GIT2TK</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, deckargenren</t>
+          <t>Italienska A: Kultur och samhälle, de italienska öarna</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -6090,14 +6090,14 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TK</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GIT2TP</t>
+          <t>GIT2TM</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Italienska A: Kultur och samhälle, mellersta Italien</t>
+          <t>Italienska A: Textanalys, en litterär resa i södra Italien</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -6137,14 +6137,14 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TM</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>GIT2TQ</t>
+          <t>GIT2TN</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, en litterär resa i mellersta Italien</t>
+          <t>Italienska A: Textanalys, deckargenren</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -6184,14 +6184,14 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TN</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GIT2Y9</t>
+          <t>GIT2TP</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2022-11-11</t>
+          <t>2021-12-21</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, familjeskildringar</t>
+          <t>Italienska A: Kultur och samhälle, mellersta Italien</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -6231,14 +6231,14 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2Y9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TP</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GIT2YA</t>
+          <t>GIT2TQ</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -6253,7 +6253,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2022-11-11</t>
+          <t>2021-12-21</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, krig och fred</t>
+          <t>Italienska A: Textanalys, en litterär resa i mellersta Italien</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6278,14 +6278,14 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TQ</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GIT2YB</t>
+          <t>GIT2Y9</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, det nya millenniets skönlitteratur</t>
+          <t>Italienska A: Textanalys, familjeskildringar</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -6325,14 +6325,14 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2Y9</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GIT2YC</t>
+          <t>GIT2YA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, 1900-talets skönlitteratur</t>
+          <t>Italienska A: Textanalys, krig och fred</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -6372,14 +6372,14 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YA</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GIT2YD</t>
+          <t>GIT2YB</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, kvinnoskildringar</t>
+          <t>Italienska A: Textanalys, det nya millenniets skönlitteratur</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -6419,19 +6419,19 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YB</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GSP39N</t>
+          <t>GIT2YC</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -6441,18 +6441,22 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
-        </is>
-      </c>
-      <c r="E136" t="inlineStr"/>
+          <t>2022-11-11</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2023-12-18</t>
+        </is>
+      </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Spanska</t>
+          <t>Italienska</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Spanska: Förberedande kurs</t>
+          <t>Italienska A: Textanalys, 1900-talets skönlitteratur</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -6462,19 +6466,19 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP39N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YC</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>GSS39S</t>
+          <t>GIT2YD</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6484,18 +6488,22 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr"/>
+          <t>2022-11-11</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2023-12-18</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk</t>
+          <t>Italienska</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Den globala skolan - undervisning inom grundskolan</t>
+          <t>Italienska A: Textanalys, kvinnoskildringar</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -6505,19 +6513,19 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YD</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>GSS39T</t>
+          <t>GIT2YE</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ITA</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -6527,18 +6535,22 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr"/>
+          <t>2022-11-11</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2023-12-18</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk</t>
+          <t>Italienska</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Den globala skolan - undervisning inom gymnasieskolan</t>
+          <t>Italienska A: Textanalys, barn- och ungdomsskildringar</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -6548,19 +6560,19 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2YE</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GSS39U</t>
+          <t>GSP39N</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -6576,12 +6588,12 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk</t>
+          <t>Spanska</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Den globala skolan - undervisning inom vuxenutbildningen</t>
+          <t>Spanska: Förberedande kurs</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6591,19 +6603,19 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP39N</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>AJP2AH</t>
+          <t>GSS39S</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -6613,18 +6625,18 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2024-04-26</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Japanska</t>
+          <t>Svenska som andraspråk</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Klassisk japanska</t>
+          <t>Den globala skolan - undervisning inom grundskolan</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -6634,19 +6646,19 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AJP2AH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39S</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GEN3BQ</t>
+          <t>GSS39T</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>ENA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -6656,18 +6668,18 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Engelska</t>
+          <t>Svenska som andraspråk</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Teman inom populärlitteraturen</t>
+          <t>Den globala skolan - undervisning inom gymnasieskolan</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -6677,19 +6689,19 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3BQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39T</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GEN3BR</t>
+          <t>GSS39U</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ENA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6699,18 +6711,18 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Engelska</t>
+          <t>Svenska som andraspråk</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Kulturella texter och kontexter</t>
+          <t>Den globala skolan - undervisning inom vuxenutbildningen</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -6720,19 +6732,19 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3BR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39U</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GSS3BN</t>
+          <t>AJP2AH</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6742,18 +6754,18 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2024-04-26</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk</t>
+          <t>Japanska</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk II med didaktisk inriktning</t>
+          <t>Klassisk japanska</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -6763,19 +6775,19 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AJP2AH</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>GKI3C9</t>
+          <t>GEN3BQ</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6785,18 +6797,18 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2024-06-19</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Kinesiska</t>
+          <t>Engelska</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Kinesiska för affärslivet II</t>
+          <t>Teman inom populärlitteraturen</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -6806,19 +6818,19 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3C9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3BQ</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>GKI3CE</t>
+          <t>GEN3BR</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6828,18 +6840,18 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2024-06-19</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Kinesiska</t>
+          <t>Engelska</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Kinesiska III med didaktisk inriktning</t>
+          <t>Kulturella texter och kontexter</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -6849,14 +6861,14 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3CE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3BR</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>GSS3C6</t>
+          <t>GSS3BN</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -6871,7 +6883,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>2024-06-19</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -6882,7 +6894,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Lärande genom fiktionstext i gymnasieskolan</t>
+          <t>Svenska som andraspråk II med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -6892,19 +6904,19 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3C6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BN</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>GFR3D2</t>
+          <t>GKI3C9</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6914,18 +6926,18 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-19</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Franska</t>
+          <t>Kinesiska</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Franska I med didaktisk inriktning</t>
+          <t>Kinesiska för affärslivet II</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -6935,19 +6947,19 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3D2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3C9</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>GFR3D3</t>
+          <t>GKI3CE</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6957,18 +6969,18 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-19</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Franska</t>
+          <t>Kinesiska</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Franska II med didaktisk inriktning</t>
+          <t>Kinesiska III med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -6978,19 +6990,19 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3D3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3CE</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GTY3CU</t>
+          <t>GSS3C6</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>TYA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7000,18 +7012,18 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-19</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Tyska</t>
+          <t>Svenska som andraspråk</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Tyska II med didaktisk inriktning</t>
+          <t>Lärande genom fiktionstext i gymnasieskolan</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -7021,14 +7033,14 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3CU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3C6</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GFR3DL</t>
+          <t>GFR3D2</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -7043,7 +7055,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2025-01-13</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
@@ -7054,7 +7066,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Franska för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i Lärarlyftet</t>
+          <t>Franska I med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -7064,19 +7076,19 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3DL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3D2</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GPR3E5</t>
+          <t>GFR3D3</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7086,18 +7098,18 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Portugisiska</t>
+          <t>Franska</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Kommunikation på arbetsplatsen: Interkulturalitet och inkludering</t>
+          <t>Franska II med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -7107,19 +7119,19 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR3E5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3D3</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GSV3FP</t>
+          <t>GTY3CU</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>SVE</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7129,18 +7141,18 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2025-05-14</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Svenska</t>
+          <t>Tyska</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Språk-, läs- och skrivutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+          <t>Tyska II med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7150,19 +7162,19 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3FP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3CU</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>AEN2BR</t>
+          <t>GFR3DL</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ENA</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7172,18 +7184,18 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>2025-01-13</t>
         </is>
       </c>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Engelska</t>
+          <t>Franska</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Interkulturella litteraturstudier: Akademisk läsning</t>
+          <t>Franska för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i Lärarlyftet</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -7193,19 +7205,19 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2BR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3DL</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>GSV3JE</t>
+          <t>GPR3E5</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SVE</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7215,18 +7227,18 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Svenska</t>
+          <t>Portugisiska</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Språk-, läs- och skrivutveckling i åldrarna 5–9 år</t>
+          <t>Kommunikation på arbetsplatsen: Interkulturalitet och inkludering</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -7236,19 +7248,19 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3JE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR3E5</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>GSS3K2</t>
+          <t>GSV3FP</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>SVE</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7258,18 +7270,18 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2025-05-14</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Svenska som andraspråk</t>
+          <t>Svenska</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Litteraturdidaktik för ämneslärare i svenska som andraspråk på gymnasial nivå</t>
+          <t>Språk-, läs- och skrivutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7279,14 +7291,14 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3K2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3FP</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GEN3K3</t>
+          <t>AEN2BR</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7301,7 +7313,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -7312,7 +7324,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Engelska II</t>
+          <t>Interkulturella litteraturstudier: Akademisk läsning</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -7322,14 +7334,14 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3K3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2BR</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>ASV2CP</t>
+          <t>GSV3JE</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -7344,7 +7356,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -7355,7 +7367,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Språk-, läs- och skrivdidaktisk fördjupning för undervisning i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+          <t>Språk-, läs- och skrivutveckling i åldrarna 5–9 år</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7365,19 +7377,19 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASV2CP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3JE</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>ASV2CQ</t>
+          <t>GSS3K2</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>SVE</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7387,18 +7399,18 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Svenska</t>
+          <t>Svenska som andraspråk</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Språk-, läs- och skrivdidaktisk fördjupning för undervisning i årskurs 4–6 utifrån första- och andraspråksperspektiv</t>
+          <t>Litteraturdidaktik för ämneslärare i svenska som andraspråk på gymnasial nivå</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -7408,14 +7420,14 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASV2CQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3K2</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>AEN2CT</t>
+          <t>GEN3K3</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -7430,7 +7442,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -7441,7 +7453,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Introduktion till interkulturella litteraturstudier</t>
+          <t>Engelska II</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -7451,19 +7463,19 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2CT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEN3K3</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>AEN2CU</t>
+          <t>ASV2CP</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>ENA</t>
+          <t>SVE</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7473,18 +7485,18 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Engelska</t>
+          <t>Svenska</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Interkulturella litteraturstudier: Magisterexamensarbete</t>
+          <t>Språk-, läs- och skrivdidaktisk fördjupning för undervisning i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -7494,19 +7506,19 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2CU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASV2CP</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GIT3KL</t>
+          <t>ASV2CQ</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>SVE</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7516,18 +7528,18 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Italienska</t>
+          <t>Svenska</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Italienska A: Textanalys, barn- och ungdomsskildringar</t>
+          <t>Språk-, läs- och skrivdidaktisk fördjupning för undervisning i årskurs 4–6 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -7537,19 +7549,19 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASV2CQ</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GIT3KM</t>
+          <t>AEN2CT</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -7565,12 +7577,12 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Italienska</t>
+          <t>Engelska</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Italienska A: Fonetik och muntlig språkfärdighet</t>
+          <t>Introduktion till interkulturella litteraturstudier</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -7580,19 +7592,19 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2CT</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GIT3KN</t>
+          <t>AEN2CU</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -7608,12 +7620,12 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Italienska</t>
+          <t>Engelska</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Italienska A: Grammatik och skriftlig språkfärdighet</t>
+          <t>Interkulturella litteraturstudier: Magisterexamensarbete</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -7623,14 +7635,14 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEN2CU</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GIT3KP</t>
+          <t>GIT3KN</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -7656,7 +7668,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Italienska B: Muntlig språkfärdighet och kulturkunskap</t>
+          <t>Italienska A: Grammatik och skriftlig språkfärdighet</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -7666,7 +7678,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KN</t>
         </is>
       </c>
     </row>

</xml_diff>